<commit_message>
feat: replace mobile navbar dropdown with bottom navigation and update database schema with calendar seeding logic
</commit_message>
<xml_diff>
--- a/Normal Service_time_tables.xlsx
+++ b/Normal Service_time_tables.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dewmina/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dewmina/devbykushan:bus-booking-app/bus-booking-app/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{241B8D5E-36C9-B84E-A4D6-B52F19110F02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{659EE45B-B378-2445-9F1E-786E94E5CA0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3980" yWindow="2780" windowWidth="28040" windowHeight="17180" xr2:uid="{47FF2829-6A9C-1D4A-81F9-56D1E767C690}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="908" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="920" uniqueCount="46">
   <si>
     <t>Date</t>
   </si>
@@ -199,9 +199,6 @@
   </si>
   <si>
     <t>12.40pm</t>
-  </si>
-  <si>
-    <t>1.40am</t>
   </si>
 </sst>
 </file>
@@ -794,10 +791,10 @@
         <v>46265</v>
       </c>
       <c r="Q7" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="R7" t="s">
-        <v>24</v>
+        <v>37</v>
       </c>
     </row>
     <row r="8" spans="5:18" x14ac:dyDescent="0.2">
@@ -820,7 +817,7 @@
         <v>46266</v>
       </c>
       <c r="Q8" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="R8" t="s">
         <v>24</v>
@@ -846,10 +843,10 @@
         <v>46267</v>
       </c>
       <c r="Q9" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="R9" t="s">
-        <v>37</v>
+        <v>24</v>
       </c>
     </row>
     <row r="10" spans="5:18" x14ac:dyDescent="0.2">
@@ -950,10 +947,10 @@
         <v>46271</v>
       </c>
       <c r="Q13" t="s">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="R13" t="s">
-        <v>24</v>
+        <v>37</v>
       </c>
     </row>
     <row r="14" spans="5:18" x14ac:dyDescent="0.2">
@@ -976,7 +973,7 @@
         <v>46272</v>
       </c>
       <c r="Q14" t="s">
-        <v>33</v>
+        <v>45</v>
       </c>
       <c r="R14" t="s">
         <v>24</v>
@@ -1002,7 +999,7 @@
         <v>46273</v>
       </c>
       <c r="Q15" t="s">
-        <v>23</v>
+        <v>33</v>
       </c>
       <c r="R15" t="s">
         <v>24</v>
@@ -1028,10 +1025,10 @@
         <v>46274</v>
       </c>
       <c r="Q16" t="s">
-        <v>37</v>
+        <v>23</v>
       </c>
       <c r="R16" t="s">
-        <v>37</v>
+        <v>24</v>
       </c>
     </row>
     <row r="17" spans="5:18" x14ac:dyDescent="0.2">
@@ -1340,10 +1337,10 @@
         <v>46286</v>
       </c>
       <c r="Q28" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="R28" t="s">
-        <v>24</v>
+        <v>37</v>
       </c>
     </row>
     <row r="29" spans="5:18" x14ac:dyDescent="0.2">
@@ -1366,7 +1363,7 @@
         <v>46287</v>
       </c>
       <c r="Q29" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="R29" t="s">
         <v>24</v>
@@ -1392,10 +1389,10 @@
         <v>46288</v>
       </c>
       <c r="Q30" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="R30" t="s">
-        <v>37</v>
+        <v>24</v>
       </c>
     </row>
     <row r="31" spans="5:18" x14ac:dyDescent="0.2">
@@ -1496,10 +1493,10 @@
         <v>46292</v>
       </c>
       <c r="Q34" t="s">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="R34" t="s">
-        <v>24</v>
+        <v>37</v>
       </c>
     </row>
     <row r="35" spans="5:18" x14ac:dyDescent="0.2">
@@ -1522,7 +1519,7 @@
         <v>46293</v>
       </c>
       <c r="Q35" t="s">
-        <v>33</v>
+        <v>45</v>
       </c>
       <c r="R35" t="s">
         <v>24</v>
@@ -1548,7 +1545,7 @@
         <v>46294</v>
       </c>
       <c r="Q36" t="s">
-        <v>23</v>
+        <v>33</v>
       </c>
       <c r="R36" t="s">
         <v>24</v>
@@ -1574,7 +1571,7 @@
         <v>46295</v>
       </c>
       <c r="Q37" t="s">
-        <v>37</v>
+        <v>23</v>
       </c>
       <c r="R37" t="s">
         <v>37</v>
@@ -1886,10 +1883,10 @@
         <v>46307</v>
       </c>
       <c r="Q49" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="R49" t="s">
-        <v>24</v>
+        <v>37</v>
       </c>
     </row>
     <row r="50" spans="5:18" x14ac:dyDescent="0.2">
@@ -1912,7 +1909,7 @@
         <v>46308</v>
       </c>
       <c r="Q50" t="s">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="R50" t="s">
         <v>24</v>
@@ -1938,10 +1935,10 @@
         <v>46309</v>
       </c>
       <c r="Q51" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="R51" t="s">
-        <v>37</v>
+        <v>24</v>
       </c>
     </row>
     <row r="52" spans="5:18" x14ac:dyDescent="0.2">
@@ -2042,10 +2039,10 @@
         <v>46313</v>
       </c>
       <c r="Q55" t="s">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="R55" t="s">
-        <v>24</v>
+        <v>37</v>
       </c>
     </row>
     <row r="56" spans="5:18" x14ac:dyDescent="0.2">
@@ -2068,7 +2065,7 @@
         <v>46314</v>
       </c>
       <c r="Q56" t="s">
-        <v>33</v>
+        <v>45</v>
       </c>
       <c r="R56" t="s">
         <v>24</v>
@@ -2094,7 +2091,7 @@
         <v>46315</v>
       </c>
       <c r="Q57" t="s">
-        <v>23</v>
+        <v>33</v>
       </c>
       <c r="R57" t="s">
         <v>24</v>
@@ -2120,10 +2117,10 @@
         <v>46316</v>
       </c>
       <c r="Q58" t="s">
-        <v>37</v>
+        <v>23</v>
       </c>
       <c r="R58" t="s">
-        <v>37</v>
+        <v>24</v>
       </c>
     </row>
     <row r="59" spans="5:18" x14ac:dyDescent="0.2">
@@ -2432,10 +2429,10 @@
         <v>46328</v>
       </c>
       <c r="Q70" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="R70" t="s">
-        <v>24</v>
+        <v>37</v>
       </c>
     </row>
     <row r="71" spans="5:18" x14ac:dyDescent="0.2">
@@ -2458,21 +2455,31 @@
         <v>46329</v>
       </c>
       <c r="Q71" t="s">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="R71" t="s">
         <v>24</v>
       </c>
     </row>
+    <row r="72" spans="5:18" x14ac:dyDescent="0.2">
+      <c r="O72" t="s">
+        <v>11</v>
+      </c>
+      <c r="P72" s="3">
+        <v>46330</v>
+      </c>
+      <c r="Q72" t="s">
+        <v>33</v>
+      </c>
+      <c r="R72" t="s">
+        <v>24</v>
+      </c>
+    </row>
     <row r="74" spans="5:18" x14ac:dyDescent="0.2">
-      <c r="P74" s="3">
-        <v>46332</v>
-      </c>
+      <c r="P74" s="3"/>
     </row>
     <row r="75" spans="5:18" x14ac:dyDescent="0.2">
-      <c r="P75" s="3">
-        <v>46333</v>
-      </c>
+      <c r="P75" s="3"/>
     </row>
     <row r="76" spans="5:18" x14ac:dyDescent="0.2">
       <c r="P76" s="3"/>
@@ -2485,7 +2492,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D02F53C-4073-0D4A-ACF0-BCF9C2BFACD0}">
-  <dimension ref="B4:R87"/>
+  <dimension ref="B4:R88"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="4" spans="2:18" ht="20" x14ac:dyDescent="0.2">
@@ -2582,10 +2589,10 @@
         <v>46274</v>
       </c>
       <c r="J8" t="s">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="K8" t="s">
-        <v>24</v>
+        <v>37</v>
       </c>
       <c r="Q8" s="8"/>
     </row>
@@ -2609,7 +2616,7 @@
         <v>46275</v>
       </c>
       <c r="J9" t="s">
-        <v>33</v>
+        <v>45</v>
       </c>
       <c r="K9" t="s">
         <v>24</v>
@@ -2637,7 +2644,7 @@
         <v>46276</v>
       </c>
       <c r="J10" t="s">
-        <v>23</v>
+        <v>33</v>
       </c>
       <c r="K10" t="s">
         <v>24</v>
@@ -2663,10 +2670,10 @@
         <v>46277</v>
       </c>
       <c r="J11" t="s">
-        <v>37</v>
+        <v>23</v>
       </c>
       <c r="K11" t="s">
-        <v>37</v>
+        <v>24</v>
       </c>
     </row>
     <row r="12" spans="2:18" x14ac:dyDescent="0.2">
@@ -2975,10 +2982,10 @@
         <v>46289</v>
       </c>
       <c r="J23" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="K23" t="s">
-        <v>24</v>
+        <v>37</v>
       </c>
     </row>
     <row r="24" spans="2:11" x14ac:dyDescent="0.2">
@@ -3001,7 +3008,7 @@
         <v>46290</v>
       </c>
       <c r="J24" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="K24" t="s">
         <v>24</v>
@@ -3027,10 +3034,10 @@
         <v>46291</v>
       </c>
       <c r="J25" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="K25" t="s">
-        <v>37</v>
+        <v>24</v>
       </c>
     </row>
     <row r="26" spans="2:11" x14ac:dyDescent="0.2">
@@ -3131,10 +3138,10 @@
         <v>46295</v>
       </c>
       <c r="J29" t="s">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="K29" t="s">
-        <v>24</v>
+        <v>37</v>
       </c>
     </row>
     <row r="30" spans="2:11" x14ac:dyDescent="0.2">
@@ -3157,7 +3164,7 @@
         <v>46296</v>
       </c>
       <c r="J30" t="s">
-        <v>33</v>
+        <v>45</v>
       </c>
       <c r="K30" t="s">
         <v>24</v>
@@ -3183,7 +3190,7 @@
         <v>46297</v>
       </c>
       <c r="J31" t="s">
-        <v>23</v>
+        <v>33</v>
       </c>
       <c r="K31" t="s">
         <v>24</v>
@@ -3209,10 +3216,10 @@
         <v>46298</v>
       </c>
       <c r="J32" t="s">
-        <v>37</v>
+        <v>23</v>
       </c>
       <c r="K32" t="s">
-        <v>37</v>
+        <v>24</v>
       </c>
     </row>
     <row r="33" spans="2:11" x14ac:dyDescent="0.2">
@@ -3312,6 +3319,12 @@
       <c r="I36" s="3">
         <v>46302</v>
       </c>
+      <c r="J36" t="s">
+        <v>26</v>
+      </c>
+      <c r="K36" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="37" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B37" t="s">
@@ -3515,10 +3528,10 @@
         <v>46310</v>
       </c>
       <c r="J44" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="K44" t="s">
-        <v>24</v>
+        <v>37</v>
       </c>
     </row>
     <row r="45" spans="2:11" x14ac:dyDescent="0.2">
@@ -3541,7 +3554,7 @@
         <v>46311</v>
       </c>
       <c r="J45" t="s">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="K45" t="s">
         <v>24</v>
@@ -3567,10 +3580,10 @@
         <v>46312</v>
       </c>
       <c r="J46" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="K46" t="s">
-        <v>37</v>
+        <v>24</v>
       </c>
     </row>
     <row r="47" spans="2:11" x14ac:dyDescent="0.2">
@@ -3671,10 +3684,10 @@
         <v>46316</v>
       </c>
       <c r="J50" t="s">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="K50" t="s">
-        <v>24</v>
+        <v>37</v>
       </c>
     </row>
     <row r="51" spans="2:11" x14ac:dyDescent="0.2">
@@ -3697,7 +3710,7 @@
         <v>46317</v>
       </c>
       <c r="J51" t="s">
-        <v>33</v>
+        <v>45</v>
       </c>
       <c r="K51" t="s">
         <v>24</v>
@@ -3723,7 +3736,7 @@
         <v>46318</v>
       </c>
       <c r="J52" t="s">
-        <v>23</v>
+        <v>33</v>
       </c>
       <c r="K52" t="s">
         <v>24</v>
@@ -3749,10 +3762,10 @@
         <v>46319</v>
       </c>
       <c r="J53" t="s">
-        <v>37</v>
+        <v>23</v>
       </c>
       <c r="K53" t="s">
-        <v>37</v>
+        <v>24</v>
       </c>
     </row>
     <row r="54" spans="2:11" x14ac:dyDescent="0.2">
@@ -3852,6 +3865,12 @@
       <c r="I57" s="3">
         <v>46323</v>
       </c>
+      <c r="J57" t="s">
+        <v>26</v>
+      </c>
+      <c r="K57" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="58" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B58" t="s">
@@ -4055,10 +4074,10 @@
         <v>46331</v>
       </c>
       <c r="J65" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="K65" t="s">
-        <v>24</v>
+        <v>37</v>
       </c>
     </row>
     <row r="66" spans="2:11" x14ac:dyDescent="0.2">
@@ -4081,7 +4100,7 @@
         <v>46332</v>
       </c>
       <c r="J66" t="s">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="K66" t="s">
         <v>24</v>
@@ -4107,10 +4126,10 @@
         <v>46333</v>
       </c>
       <c r="J67" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="K67" t="s">
-        <v>37</v>
+        <v>24</v>
       </c>
     </row>
     <row r="68" spans="2:11" x14ac:dyDescent="0.2">
@@ -4211,10 +4230,10 @@
         <v>46337</v>
       </c>
       <c r="J71" t="s">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="K71" t="s">
-        <v>24</v>
+        <v>37</v>
       </c>
     </row>
     <row r="72" spans="2:11" x14ac:dyDescent="0.2">
@@ -4237,7 +4256,7 @@
         <v>46338</v>
       </c>
       <c r="J72" t="s">
-        <v>33</v>
+        <v>45</v>
       </c>
       <c r="K72" t="s">
         <v>24</v>
@@ -4263,7 +4282,7 @@
         <v>46339</v>
       </c>
       <c r="J73" t="s">
-        <v>23</v>
+        <v>33</v>
       </c>
       <c r="K73" t="s">
         <v>24</v>
@@ -4289,10 +4308,10 @@
         <v>46340</v>
       </c>
       <c r="J74" t="s">
-        <v>37</v>
+        <v>23</v>
       </c>
       <c r="K74" t="s">
-        <v>37</v>
+        <v>24</v>
       </c>
     </row>
     <row r="75" spans="2:11" x14ac:dyDescent="0.2">
@@ -4392,6 +4411,12 @@
       <c r="I78" s="3">
         <v>46344</v>
       </c>
+      <c r="J78" t="s">
+        <v>26</v>
+      </c>
+      <c r="K78" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="79" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B79" t="s">
@@ -4595,10 +4620,10 @@
         <v>46352</v>
       </c>
       <c r="J86" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="K86" t="s">
-        <v>24</v>
+        <v>37</v>
       </c>
     </row>
     <row r="87" spans="2:11" x14ac:dyDescent="0.2">
@@ -4621,13 +4646,28 @@
         <v>46353</v>
       </c>
       <c r="J87" t="s">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="K87" t="s">
         <v>24</v>
       </c>
     </row>
+    <row r="88" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="H88" t="s">
+        <v>7</v>
+      </c>
+      <c r="I88" s="3">
+        <v>46354</v>
+      </c>
+      <c r="J88" t="s">
+        <v>33</v>
+      </c>
+      <c r="K88" t="s">
+        <v>24</v>
+      </c>
+    </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>